<commit_message>
FT Durchläufe + Vergleichsskript fix
Durchläufe FT Modelle inkl. neuem Energieverbrauch
Anpassungen am Vergleichsskript für neue Benenung der Ordner
Durchlauf Vergleichsskript_neue_Nomenklatur
</commit_message>
<xml_diff>
--- a/Fischer_Tropsch/Höchst_FischerTropsch_1_Naphta_Greenfield/Datenbank.xlsx
+++ b/Fischer_Tropsch/Höchst_FischerTropsch_1_Naphta_Greenfield/Datenbank.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hem38994\Documents\GitHub\FENES_P2X\Fischer_Tropsch\Höchst_1_FischerTropsch_Naphta_Greenfield\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hem38994\Documents\GitHub\FENES_P2X\Fischer_Tropsch\Höchst_FischerTropsch_1_Naphta_Greenfield\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39AD49FB-64BE-4D6E-8871-DE8A28F17E60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D41330CD-57F0-4A3F-8A49-07F99AB8A2AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-4455" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1440" yWindow="2700" windowWidth="21600" windowHeight="10980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datenauswahl" sheetId="1" r:id="rId1"/>
@@ -1718,6 +1718,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1727,13 +1730,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1742,17 +1742,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1766,8 +1757,17 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2413,7 +2413,7 @@
         <v>329</v>
       </c>
       <c r="E8" s="66">
-        <v>38.99</v>
+        <v>10</v>
       </c>
       <c r="F8" s="35" t="s">
         <v>340</v>
@@ -3566,10 +3566,10 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="87" t="s">
+      <c r="A2" s="88" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="89" t="s">
+      <c r="B2" s="90" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="26" t="s">
@@ -3584,7 +3584,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="88"/>
+      <c r="A3" s="89"/>
       <c r="B3" s="85"/>
       <c r="C3" s="13" t="s">
         <v>107</v>
@@ -3598,7 +3598,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="88"/>
+      <c r="A4" s="89"/>
       <c r="B4" s="85"/>
       <c r="C4" s="13" t="s">
         <v>84</v>
@@ -3612,7 +3612,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="88"/>
+      <c r="A5" s="89"/>
       <c r="B5" s="85"/>
       <c r="C5" s="13" t="s">
         <v>138</v>
@@ -3626,7 +3626,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="88"/>
+      <c r="A6" s="89"/>
       <c r="B6" s="85"/>
       <c r="C6" s="13" t="s">
         <v>141</v>
@@ -3640,7 +3640,7 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="88"/>
+      <c r="A7" s="89"/>
       <c r="B7" s="85"/>
       <c r="C7" s="13" t="s">
         <v>155</v>
@@ -3654,7 +3654,7 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="88"/>
+      <c r="A8" s="89"/>
       <c r="B8" s="85"/>
       <c r="C8" s="13" t="s">
         <v>196</v>
@@ -3668,7 +3668,7 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="88"/>
+      <c r="A9" s="89"/>
       <c r="B9" s="85"/>
       <c r="C9" s="13" t="s">
         <v>167</v>
@@ -3682,7 +3682,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="88"/>
+      <c r="A10" s="89"/>
       <c r="B10" s="85"/>
       <c r="C10" s="13" t="s">
         <v>188</v>
@@ -3696,13 +3696,13 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="88"/>
+      <c r="A11" s="89"/>
       <c r="B11" s="85"/>
       <c r="E11" s="33"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="88"/>
-      <c r="B12" s="90" t="s">
+      <c r="A12" s="89"/>
+      <c r="B12" s="100" t="s">
         <v>360</v>
       </c>
       <c r="C12" s="35" t="s">
@@ -3717,7 +3717,7 @@
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="88"/>
+      <c r="A13" s="89"/>
       <c r="B13" s="91"/>
       <c r="C13" s="13" t="s">
         <v>359</v>
@@ -3731,7 +3731,7 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="88"/>
+      <c r="A14" s="89"/>
       <c r="B14" s="91"/>
       <c r="C14" s="13" t="s">
         <v>376</v>
@@ -3745,7 +3745,7 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="88"/>
+      <c r="A15" s="89"/>
       <c r="B15" s="91"/>
       <c r="C15" s="13" t="s">
         <v>139</v>
@@ -3759,7 +3759,7 @@
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="88"/>
+      <c r="A16" s="89"/>
       <c r="B16" s="91"/>
       <c r="C16" s="13" t="s">
         <v>236</v>
@@ -3773,7 +3773,7 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="88"/>
+      <c r="A17" s="89"/>
       <c r="B17" s="91"/>
       <c r="C17" s="13" t="s">
         <v>84</v>
@@ -3787,7 +3787,7 @@
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="88"/>
+      <c r="A18" s="89"/>
       <c r="B18" s="91"/>
       <c r="C18" s="13" t="s">
         <v>141</v>
@@ -3801,7 +3801,7 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="88"/>
+      <c r="A19" s="89"/>
       <c r="B19" s="91"/>
       <c r="C19" s="13" t="s">
         <v>155</v>
@@ -3815,7 +3815,7 @@
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="88"/>
+      <c r="A20" s="89"/>
       <c r="B20" s="91"/>
       <c r="C20" s="13" t="s">
         <v>196</v>
@@ -3829,7 +3829,7 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="88"/>
+      <c r="A21" s="89"/>
       <c r="B21" s="91"/>
       <c r="C21" s="13" t="s">
         <v>167</v>
@@ -3843,7 +3843,7 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="88"/>
+      <c r="A22" s="89"/>
       <c r="B22" s="91"/>
       <c r="C22" s="13" t="s">
         <v>188</v>
@@ -3857,15 +3857,15 @@
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="88"/>
-      <c r="B23" s="92"/>
+      <c r="A23" s="89"/>
+      <c r="B23" s="101"/>
       <c r="C23" s="36"/>
       <c r="D23" s="36"/>
       <c r="E23" s="37"/>
       <c r="F23" s="36"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="88"/>
+      <c r="A24" s="89"/>
       <c r="B24" s="84" t="s">
         <v>260</v>
       </c>
@@ -3881,7 +3881,7 @@
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="88"/>
+      <c r="A25" s="89"/>
       <c r="B25" s="85"/>
       <c r="C25" s="13" t="s">
         <v>107</v>
@@ -3895,7 +3895,7 @@
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="88"/>
+      <c r="A26" s="89"/>
       <c r="B26" s="85"/>
       <c r="C26" s="13" t="s">
         <v>84</v>
@@ -3909,7 +3909,7 @@
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="88"/>
+      <c r="A27" s="89"/>
       <c r="B27" s="85"/>
       <c r="C27" s="13" t="s">
         <v>281</v>
@@ -3923,7 +3923,7 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="88"/>
+      <c r="A28" s="89"/>
       <c r="B28" s="85"/>
       <c r="C28" s="13" t="s">
         <v>141</v>
@@ -3937,7 +3937,7 @@
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="88"/>
+      <c r="A29" s="89"/>
       <c r="B29" s="85"/>
       <c r="C29" s="13" t="s">
         <v>155</v>
@@ -3951,7 +3951,7 @@
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="88"/>
+      <c r="A30" s="89"/>
       <c r="B30" s="85"/>
       <c r="C30" s="13" t="s">
         <v>196</v>
@@ -3965,7 +3965,7 @@
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="88"/>
+      <c r="A31" s="89"/>
       <c r="B31" s="85"/>
       <c r="C31" s="13" t="s">
         <v>167</v>
@@ -3979,7 +3979,7 @@
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="88"/>
+      <c r="A32" s="89"/>
       <c r="B32" s="85"/>
       <c r="C32" s="13" t="s">
         <v>188</v>
@@ -3993,7 +3993,7 @@
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="88"/>
+      <c r="A33" s="89"/>
       <c r="B33" s="86"/>
       <c r="C33" s="36"/>
       <c r="D33" s="36"/>
@@ -4001,7 +4001,7 @@
       <c r="F33" s="36"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="88"/>
+      <c r="A34" s="89"/>
       <c r="B34" s="83" t="s">
         <v>227</v>
       </c>
@@ -4017,7 +4017,7 @@
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="88"/>
+      <c r="A35" s="89"/>
       <c r="B35" s="83"/>
       <c r="C35" s="13" t="s">
         <v>107</v>
@@ -4031,7 +4031,7 @@
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="88"/>
+      <c r="A36" s="89"/>
       <c r="B36" s="83"/>
       <c r="C36" s="13" t="s">
         <v>84</v>
@@ -4045,7 +4045,7 @@
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="88"/>
+      <c r="A37" s="89"/>
       <c r="B37" s="83"/>
       <c r="C37" s="13" t="s">
         <v>268</v>
@@ -4059,7 +4059,7 @@
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="88"/>
+      <c r="A38" s="89"/>
       <c r="B38" s="83"/>
       <c r="C38" s="13" t="s">
         <v>246</v>
@@ -4073,7 +4073,7 @@
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="88"/>
+      <c r="A39" s="89"/>
       <c r="B39" s="83"/>
       <c r="C39" s="13" t="s">
         <v>141</v>
@@ -4087,7 +4087,7 @@
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="88"/>
+      <c r="A40" s="89"/>
       <c r="B40" s="83"/>
       <c r="C40" s="13" t="s">
         <v>155</v>
@@ -4101,7 +4101,7 @@
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="88"/>
+      <c r="A41" s="89"/>
       <c r="B41" s="83"/>
       <c r="C41" s="13" t="s">
         <v>196</v>
@@ -4115,7 +4115,7 @@
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="88"/>
+      <c r="A42" s="89"/>
       <c r="B42" s="83"/>
       <c r="C42" s="13" t="s">
         <v>167</v>
@@ -4129,7 +4129,7 @@
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="88"/>
+      <c r="A43" s="89"/>
       <c r="B43" s="83"/>
       <c r="C43" s="13" t="s">
         <v>188</v>
@@ -4143,15 +4143,15 @@
       </c>
     </row>
     <row r="44" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="88"/>
+      <c r="A44" s="89"/>
       <c r="B44" s="83"/>
       <c r="E44" s="33"/>
     </row>
     <row r="45" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="87" t="s">
+      <c r="A45" s="88" t="s">
         <v>71</v>
       </c>
-      <c r="B45" s="96" t="s">
+      <c r="B45" s="103" t="s">
         <v>3</v>
       </c>
       <c r="C45" s="26" t="s">
@@ -4166,7 +4166,7 @@
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="88"/>
+      <c r="A46" s="89"/>
       <c r="B46" s="83"/>
       <c r="C46" s="13" t="s">
         <v>111</v>
@@ -4180,7 +4180,7 @@
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="88"/>
+      <c r="A47" s="89"/>
       <c r="B47" s="83"/>
       <c r="C47" s="13" t="s">
         <v>135</v>
@@ -4194,7 +4194,7 @@
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="88"/>
+      <c r="A48" s="89"/>
       <c r="B48" s="83"/>
       <c r="C48" s="13" t="s">
         <v>136</v>
@@ -4208,7 +4208,7 @@
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="88"/>
+      <c r="A49" s="89"/>
       <c r="B49" s="83"/>
       <c r="C49" s="13" t="s">
         <v>141</v>
@@ -4222,7 +4222,7 @@
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="88"/>
+      <c r="A50" s="89"/>
       <c r="B50" s="83"/>
       <c r="C50" s="13" t="s">
         <v>155</v>
@@ -4236,7 +4236,7 @@
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" s="88"/>
+      <c r="A51" s="89"/>
       <c r="B51" s="83"/>
       <c r="C51" s="13" t="s">
         <v>196</v>
@@ -4250,7 +4250,7 @@
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="88"/>
+      <c r="A52" s="89"/>
       <c r="B52" s="83"/>
       <c r="C52" s="13" t="s">
         <v>167</v>
@@ -4264,7 +4264,7 @@
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="88"/>
+      <c r="A53" s="89"/>
       <c r="B53" s="83"/>
       <c r="C53" s="13" t="s">
         <v>188</v>
@@ -4278,15 +4278,15 @@
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A54" s="88"/>
-      <c r="B54" s="97"/>
+      <c r="A54" s="89"/>
+      <c r="B54" s="95"/>
       <c r="C54" s="36"/>
       <c r="D54" s="36"/>
       <c r="E54" s="37"/>
       <c r="F54" s="36"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="88"/>
+      <c r="A55" s="89"/>
       <c r="B55" s="83" t="s">
         <v>301</v>
       </c>
@@ -4302,7 +4302,7 @@
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="88"/>
+      <c r="A56" s="89"/>
       <c r="B56" s="83"/>
       <c r="C56" s="13" t="s">
         <v>111</v>
@@ -4316,7 +4316,7 @@
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="88"/>
+      <c r="A57" s="89"/>
       <c r="B57" s="83"/>
       <c r="C57" s="13" t="s">
         <v>135</v>
@@ -4330,7 +4330,7 @@
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="88"/>
+      <c r="A58" s="89"/>
       <c r="B58" s="83"/>
       <c r="C58" s="13" t="s">
         <v>136</v>
@@ -4344,7 +4344,7 @@
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" s="88"/>
+      <c r="A59" s="89"/>
       <c r="B59" s="83"/>
       <c r="C59" s="13" t="s">
         <v>141</v>
@@ -4358,7 +4358,7 @@
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A60" s="88"/>
+      <c r="A60" s="89"/>
       <c r="B60" s="83"/>
       <c r="C60" s="13" t="s">
         <v>155</v>
@@ -4372,7 +4372,7 @@
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A61" s="88"/>
+      <c r="A61" s="89"/>
       <c r="B61" s="83"/>
       <c r="C61" s="13" t="s">
         <v>196</v>
@@ -4386,7 +4386,7 @@
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" s="88"/>
+      <c r="A62" s="89"/>
       <c r="B62" s="83"/>
       <c r="C62" s="13" t="s">
         <v>167</v>
@@ -4400,7 +4400,7 @@
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" s="88"/>
+      <c r="A63" s="89"/>
       <c r="B63" s="83"/>
       <c r="C63" s="13" t="s">
         <v>188</v>
@@ -4414,12 +4414,12 @@
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A64" s="88"/>
-      <c r="B64" s="97"/>
+      <c r="A64" s="89"/>
+      <c r="B64" s="95"/>
       <c r="E64" s="33"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A65" s="88"/>
+      <c r="A65" s="89"/>
       <c r="B65" s="94" t="s">
         <v>6</v>
       </c>
@@ -4435,7 +4435,7 @@
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A66" s="88"/>
+      <c r="A66" s="89"/>
       <c r="B66" s="83"/>
       <c r="C66" s="13" t="s">
         <v>113</v>
@@ -4449,7 +4449,7 @@
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A67" s="88"/>
+      <c r="A67" s="89"/>
       <c r="B67" s="85"/>
       <c r="C67" s="13" t="s">
         <v>111</v>
@@ -4463,7 +4463,7 @@
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68" s="88"/>
+      <c r="A68" s="89"/>
       <c r="B68" s="85"/>
       <c r="C68" s="13" t="s">
         <v>107</v>
@@ -4477,7 +4477,7 @@
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A69" s="88"/>
+      <c r="A69" s="89"/>
       <c r="B69" s="85"/>
       <c r="C69" s="13" t="s">
         <v>126</v>
@@ -4491,7 +4491,7 @@
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A70" s="88"/>
+      <c r="A70" s="89"/>
       <c r="B70" s="85"/>
       <c r="C70" s="13" t="s">
         <v>127</v>
@@ -4505,7 +4505,7 @@
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A71" s="88"/>
+      <c r="A71" s="89"/>
       <c r="B71" s="85"/>
       <c r="C71" s="13" t="s">
         <v>141</v>
@@ -4519,7 +4519,7 @@
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A72" s="88"/>
+      <c r="A72" s="89"/>
       <c r="B72" s="85"/>
       <c r="C72" s="13" t="s">
         <v>155</v>
@@ -4533,7 +4533,7 @@
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A73" s="88"/>
+      <c r="A73" s="89"/>
       <c r="B73" s="85"/>
       <c r="C73" s="13" t="s">
         <v>196</v>
@@ -4547,7 +4547,7 @@
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A74" s="88"/>
+      <c r="A74" s="89"/>
       <c r="B74" s="85"/>
       <c r="C74" s="13" t="s">
         <v>167</v>
@@ -4561,7 +4561,7 @@
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A75" s="88"/>
+      <c r="A75" s="89"/>
       <c r="B75" s="85"/>
       <c r="C75" s="13" t="s">
         <v>188</v>
@@ -4576,17 +4576,17 @@
     </row>
     <row r="76" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A76" s="93"/>
-      <c r="B76" s="95"/>
+      <c r="B76" s="102"/>
       <c r="C76" s="40"/>
       <c r="D76" s="40"/>
       <c r="E76" s="41"/>
       <c r="F76" s="40"/>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A77" s="87" t="s">
+      <c r="A77" s="88" t="s">
         <v>72</v>
       </c>
-      <c r="B77" s="89" t="s">
+      <c r="B77" s="90" t="s">
         <v>73</v>
       </c>
       <c r="C77" s="26" t="s">
@@ -4601,7 +4601,7 @@
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A78" s="88"/>
+      <c r="A78" s="89"/>
       <c r="B78" s="85"/>
       <c r="C78" s="13" t="s">
         <v>153</v>
@@ -4615,12 +4615,12 @@
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" s="88"/>
+      <c r="A79" s="89"/>
       <c r="B79" s="86"/>
       <c r="E79" s="31"/>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A80" s="88"/>
+      <c r="A80" s="89"/>
       <c r="B80" s="94" t="s">
         <v>4</v>
       </c>
@@ -4636,7 +4636,7 @@
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A81" s="88"/>
+      <c r="A81" s="89"/>
       <c r="B81" s="83"/>
       <c r="C81" s="13" t="s">
         <v>107</v>
@@ -4650,7 +4650,7 @@
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A82" s="88"/>
+      <c r="A82" s="89"/>
       <c r="B82" s="83"/>
       <c r="C82" s="13" t="s">
         <v>122</v>
@@ -4664,7 +4664,7 @@
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A83" s="88"/>
+      <c r="A83" s="89"/>
       <c r="B83" s="83"/>
       <c r="C83" s="13" t="s">
         <v>141</v>
@@ -4678,7 +4678,7 @@
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A84" s="88"/>
+      <c r="A84" s="89"/>
       <c r="B84" s="83"/>
       <c r="C84" s="13" t="s">
         <v>155</v>
@@ -4692,7 +4692,7 @@
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A85" s="88"/>
+      <c r="A85" s="89"/>
       <c r="B85" s="83"/>
       <c r="C85" s="13" t="s">
         <v>161</v>
@@ -4706,7 +4706,7 @@
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A86" s="88"/>
+      <c r="A86" s="89"/>
       <c r="B86" s="83"/>
       <c r="C86" s="13" t="s">
         <v>196</v>
@@ -4720,7 +4720,7 @@
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A87" s="88"/>
+      <c r="A87" s="89"/>
       <c r="B87" s="83"/>
       <c r="C87" s="13" t="s">
         <v>167</v>
@@ -4734,7 +4734,7 @@
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A88" s="88"/>
+      <c r="A88" s="89"/>
       <c r="B88" s="83"/>
       <c r="C88" s="13" t="s">
         <v>188</v>
@@ -4748,11 +4748,11 @@
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A89" s="88"/>
-      <c r="B89" s="97"/>
+      <c r="A89" s="89"/>
+      <c r="B89" s="95"/>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A90" s="88"/>
+      <c r="A90" s="89"/>
       <c r="B90" s="94" t="s">
         <v>5</v>
       </c>
@@ -4768,7 +4768,7 @@
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A91" s="88"/>
+      <c r="A91" s="89"/>
       <c r="B91" s="83"/>
       <c r="C91" s="13" t="s">
         <v>108</v>
@@ -4782,7 +4782,7 @@
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A92" s="88"/>
+      <c r="A92" s="89"/>
       <c r="B92" s="83"/>
       <c r="C92" s="13" t="s">
         <v>120</v>
@@ -4796,7 +4796,7 @@
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A93" s="88"/>
+      <c r="A93" s="89"/>
       <c r="B93" s="83"/>
       <c r="C93" s="13" t="s">
         <v>141</v>
@@ -4810,7 +4810,7 @@
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A94" s="88"/>
+      <c r="A94" s="89"/>
       <c r="B94" s="83"/>
       <c r="C94" s="13" t="s">
         <v>155</v>
@@ -4824,7 +4824,7 @@
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A95" s="88"/>
+      <c r="A95" s="89"/>
       <c r="B95" s="83"/>
       <c r="C95" s="13" t="s">
         <v>161</v>
@@ -4838,7 +4838,7 @@
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A96" s="88"/>
+      <c r="A96" s="89"/>
       <c r="B96" s="83"/>
       <c r="C96" s="13" t="s">
         <v>196</v>
@@ -4852,7 +4852,7 @@
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A97" s="88"/>
+      <c r="A97" s="89"/>
       <c r="B97" s="83"/>
       <c r="C97" s="13" t="s">
         <v>167</v>
@@ -4866,7 +4866,7 @@
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A98" s="88"/>
+      <c r="A98" s="89"/>
       <c r="B98" s="83"/>
       <c r="C98" s="13" t="s">
         <v>188</v>
@@ -4881,13 +4881,13 @@
     </row>
     <row r="99" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A99" s="93"/>
-      <c r="B99" s="99"/>
+      <c r="B99" s="96"/>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A100" s="87" t="s">
+      <c r="A100" s="88" t="s">
         <v>76</v>
       </c>
-      <c r="B100" s="89" t="s">
+      <c r="B100" s="90" t="s">
         <v>73</v>
       </c>
       <c r="C100" s="26" t="s">
@@ -4902,7 +4902,7 @@
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A101" s="88"/>
+      <c r="A101" s="89"/>
       <c r="B101" s="85"/>
       <c r="C101" s="13" t="s">
         <v>150</v>
@@ -4916,7 +4916,7 @@
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A102" s="88"/>
+      <c r="A102" s="89"/>
       <c r="B102" s="86"/>
       <c r="C102" s="36"/>
       <c r="D102" s="36"/>
@@ -4924,7 +4924,7 @@
       <c r="F102" s="36"/>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A103" s="88"/>
+      <c r="A103" s="89"/>
       <c r="B103" s="84" t="s">
         <v>290</v>
       </c>
@@ -4940,7 +4940,7 @@
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A104" s="88"/>
+      <c r="A104" s="89"/>
       <c r="B104" s="85"/>
       <c r="C104" s="13" t="s">
         <v>294</v>
@@ -4954,12 +4954,12 @@
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A105" s="88"/>
+      <c r="A105" s="89"/>
       <c r="B105" s="86"/>
       <c r="E105" s="33"/>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A106" s="88"/>
+      <c r="A106" s="89"/>
       <c r="B106" s="84" t="s">
         <v>79</v>
       </c>
@@ -4975,7 +4975,7 @@
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A107" s="88"/>
+      <c r="A107" s="89"/>
       <c r="B107" s="85"/>
       <c r="C107" s="13" t="s">
         <v>151</v>
@@ -4989,7 +4989,7 @@
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A108" s="88"/>
+      <c r="A108" s="89"/>
       <c r="B108" s="86"/>
       <c r="C108" s="36"/>
       <c r="D108" s="36"/>
@@ -4997,8 +4997,8 @@
       <c r="F108" s="36"/>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A109" s="88"/>
-      <c r="B109" s="100" t="s">
+      <c r="A109" s="89"/>
+      <c r="B109" s="97" t="s">
         <v>367</v>
       </c>
       <c r="C109" s="35" t="s">
@@ -5013,8 +5013,8 @@
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A110" s="88"/>
-      <c r="B110" s="101"/>
+      <c r="A110" s="89"/>
+      <c r="B110" s="98"/>
       <c r="C110" s="13" t="s">
         <v>372</v>
       </c>
@@ -5027,15 +5027,15 @@
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A111" s="88"/>
-      <c r="B111" s="102"/>
+      <c r="A111" s="89"/>
+      <c r="B111" s="99"/>
       <c r="C111" s="36"/>
       <c r="D111" s="36"/>
       <c r="E111" s="37"/>
       <c r="F111" s="36"/>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A112" s="88"/>
+      <c r="A112" s="89"/>
       <c r="B112" s="91" t="s">
         <v>327</v>
       </c>
@@ -5051,7 +5051,7 @@
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A113" s="88"/>
+      <c r="A113" s="89"/>
       <c r="B113" s="91"/>
       <c r="C113" s="13" t="s">
         <v>358</v>
@@ -5066,17 +5066,17 @@
     </row>
     <row r="114" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A114" s="93"/>
-      <c r="B114" s="98"/>
+      <c r="B114" s="92"/>
       <c r="C114" s="40"/>
       <c r="D114" s="40"/>
       <c r="E114" s="41"/>
       <c r="F114" s="40"/>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A115" s="87" t="s">
+      <c r="A115" s="88" t="s">
         <v>163</v>
       </c>
-      <c r="B115" s="89" t="s">
+      <c r="B115" s="90" t="s">
         <v>13</v>
       </c>
       <c r="C115" s="26" t="s">
@@ -5091,7 +5091,7 @@
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A116" s="88"/>
+      <c r="A116" s="89"/>
       <c r="B116" s="85"/>
       <c r="C116" s="13" t="s">
         <v>174</v>
@@ -5104,7 +5104,7 @@
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A117" s="88"/>
+      <c r="A117" s="89"/>
       <c r="B117" s="86"/>
       <c r="C117" s="36"/>
       <c r="D117" s="36"/>
@@ -5112,7 +5112,7 @@
       <c r="F117" s="36"/>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A118" s="88"/>
+      <c r="A118" s="89"/>
       <c r="B118" s="84" t="s">
         <v>183</v>
       </c>
@@ -5127,7 +5127,7 @@
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A119" s="88"/>
+      <c r="A119" s="89"/>
       <c r="B119" s="85"/>
       <c r="C119" s="13" t="s">
         <v>181</v>
@@ -5140,7 +5140,7 @@
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A120" s="88"/>
+      <c r="A120" s="89"/>
       <c r="B120" s="85"/>
       <c r="C120" s="13" t="s">
         <v>177</v>
@@ -5153,7 +5153,7 @@
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A121" s="88"/>
+      <c r="A121" s="89"/>
       <c r="B121" s="85"/>
       <c r="C121" s="13" t="s">
         <v>179</v>
@@ -5166,7 +5166,7 @@
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A122" s="88"/>
+      <c r="A122" s="89"/>
       <c r="B122" s="85"/>
       <c r="C122" s="13" t="s">
         <v>182</v>
@@ -5179,7 +5179,7 @@
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A123" s="88"/>
+      <c r="A123" s="89"/>
       <c r="B123" s="85"/>
       <c r="C123" s="13" t="s">
         <v>191</v>
@@ -5192,11 +5192,11 @@
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A124" s="88"/>
+      <c r="A124" s="89"/>
       <c r="B124" s="86"/>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A125" s="88"/>
+      <c r="A125" s="89"/>
       <c r="B125" s="84" t="s">
         <v>206</v>
       </c>
@@ -5212,7 +5212,7 @@
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A126" s="88"/>
+      <c r="A126" s="89"/>
       <c r="B126" s="85"/>
       <c r="C126" s="13" t="s">
         <v>204</v>
@@ -5225,7 +5225,7 @@
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A127" s="88"/>
+      <c r="A127" s="89"/>
       <c r="B127" s="85"/>
       <c r="C127" s="13" t="s">
         <v>215</v>
@@ -5238,7 +5238,7 @@
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A128" s="88"/>
+      <c r="A128" s="89"/>
       <c r="B128" s="85"/>
       <c r="C128" s="13" t="s">
         <v>205</v>
@@ -5251,7 +5251,7 @@
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A129" s="88"/>
+      <c r="A129" s="89"/>
       <c r="B129" s="85"/>
       <c r="C129" s="13" t="s">
         <v>296</v>
@@ -5264,7 +5264,7 @@
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A130" s="88"/>
+      <c r="A130" s="89"/>
       <c r="B130" s="85"/>
       <c r="C130" s="44" t="s">
         <v>320</v>
@@ -5278,7 +5278,7 @@
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A131" s="88"/>
+      <c r="A131" s="89"/>
       <c r="B131" s="85"/>
       <c r="C131" s="44" t="s">
         <v>322</v>
@@ -5292,7 +5292,7 @@
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A132" s="88"/>
+      <c r="A132" s="89"/>
       <c r="B132" s="85"/>
       <c r="C132" s="13" t="s">
         <v>217</v>
@@ -5305,7 +5305,7 @@
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A133" s="88"/>
+      <c r="A133" s="89"/>
       <c r="B133" s="85"/>
       <c r="C133" s="13" t="s">
         <v>221</v>
@@ -5318,7 +5318,7 @@
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A134" s="88"/>
+      <c r="A134" s="89"/>
       <c r="B134" s="85"/>
       <c r="C134" s="13" t="s">
         <v>202</v>
@@ -5331,7 +5331,7 @@
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A135" s="88"/>
+      <c r="A135" s="89"/>
       <c r="B135" s="85"/>
       <c r="C135" s="44" t="s">
         <v>247</v>
@@ -5345,7 +5345,7 @@
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A136" s="88"/>
+      <c r="A136" s="89"/>
       <c r="B136" s="85"/>
       <c r="C136" s="44" t="s">
         <v>379</v>
@@ -5359,7 +5359,7 @@
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A137" s="88"/>
+      <c r="A137" s="89"/>
       <c r="B137" s="85"/>
       <c r="C137" s="44" t="s">
         <v>361</v>
@@ -5373,7 +5373,7 @@
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A138" s="88"/>
+      <c r="A138" s="89"/>
       <c r="B138" s="85"/>
       <c r="C138" s="44" t="s">
         <v>381</v>
@@ -5387,7 +5387,7 @@
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A139" s="88"/>
+      <c r="A139" s="89"/>
       <c r="B139" s="86"/>
       <c r="C139" s="44"/>
       <c r="D139" s="44"/>
@@ -5395,7 +5395,7 @@
       <c r="F139" s="44"/>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A140" s="88"/>
+      <c r="A140" s="89"/>
       <c r="B140" s="84" t="s">
         <v>222</v>
       </c>
@@ -5411,7 +5411,7 @@
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A141" s="88"/>
+      <c r="A141" s="89"/>
       <c r="B141" s="85"/>
       <c r="C141" s="13" t="s">
         <v>298</v>
@@ -5424,7 +5424,7 @@
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A142" s="88"/>
+      <c r="A142" s="89"/>
       <c r="B142" s="85"/>
       <c r="C142" s="13" t="s">
         <v>225</v>
@@ -5437,7 +5437,7 @@
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A143" s="88"/>
+      <c r="A143" s="89"/>
       <c r="B143" s="85"/>
       <c r="C143" s="44" t="s">
         <v>249</v>
@@ -5451,7 +5451,7 @@
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A144" s="88"/>
+      <c r="A144" s="89"/>
       <c r="B144" s="85"/>
       <c r="C144" s="44" t="s">
         <v>362</v>
@@ -5465,7 +5465,7 @@
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A145" s="88"/>
+      <c r="A145" s="89"/>
       <c r="B145" s="86"/>
       <c r="C145" s="36"/>
       <c r="D145" s="36"/>
@@ -5473,8 +5473,8 @@
       <c r="F145" s="36"/>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A146" s="88"/>
-      <c r="B146" s="103" t="s">
+      <c r="A146" s="89"/>
+      <c r="B146" s="87" t="s">
         <v>382</v>
       </c>
       <c r="C146" s="13" t="s">
@@ -5488,8 +5488,8 @@
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A147" s="88"/>
-      <c r="B147" s="103"/>
+      <c r="A147" s="89"/>
+      <c r="B147" s="87"/>
       <c r="C147" s="13" t="s">
         <v>384</v>
       </c>
@@ -5502,12 +5502,15 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="B140:B145"/>
-    <mergeCell ref="B146:B147"/>
-    <mergeCell ref="A115:A147"/>
-    <mergeCell ref="B115:B117"/>
-    <mergeCell ref="B125:B139"/>
-    <mergeCell ref="B118:B124"/>
+    <mergeCell ref="A2:A44"/>
+    <mergeCell ref="B2:B11"/>
+    <mergeCell ref="B12:B23"/>
+    <mergeCell ref="B34:B44"/>
+    <mergeCell ref="A45:A76"/>
+    <mergeCell ref="B65:B76"/>
+    <mergeCell ref="B24:B33"/>
+    <mergeCell ref="B45:B54"/>
+    <mergeCell ref="B55:B64"/>
     <mergeCell ref="B112:B114"/>
     <mergeCell ref="B77:B79"/>
     <mergeCell ref="A77:A99"/>
@@ -5518,15 +5521,12 @@
     <mergeCell ref="B103:B105"/>
     <mergeCell ref="B106:B108"/>
     <mergeCell ref="B109:B111"/>
-    <mergeCell ref="A2:A44"/>
-    <mergeCell ref="B2:B11"/>
-    <mergeCell ref="B12:B23"/>
-    <mergeCell ref="B34:B44"/>
-    <mergeCell ref="A45:A76"/>
-    <mergeCell ref="B65:B76"/>
-    <mergeCell ref="B24:B33"/>
-    <mergeCell ref="B45:B54"/>
-    <mergeCell ref="B55:B64"/>
+    <mergeCell ref="B140:B145"/>
+    <mergeCell ref="B146:B147"/>
+    <mergeCell ref="A115:A147"/>
+    <mergeCell ref="B115:B117"/>
+    <mergeCell ref="B125:B139"/>
+    <mergeCell ref="B118:B124"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>